<commit_message>
Reschedule STEP 1 to TAF end date (Sep 2027): PIN by May 2027, pipeline target Sep 2027
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tt9bQwcKRKX4vaP5NybJqL
</commit_message>
<xml_diff>
--- a/hutan-desa-pasir/Milestone_Matrix_HD_Pasir_PVClimate.xlsx
+++ b/hutan-desa-pasir/Milestone_Matrix_HD_Pasir_PVClimate.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Plan Vivo PV Climate · STEP 1 = SETAPAK 4 (M1–M7) · STEP 2 = Post-SETAPAK 4 (M8–M12) · Bulan 1 = Oktober 2026</t>
+          <t>Plan Vivo PV Climate · STEP 1 = SETAPAK 4 (M1–M7, Okt 2026–Sep 2027) · STEP 2 = Post-SETAPAK 4 (M8–M12) · Bulan 1 = Oktober 2026</t>
         </is>
       </c>
     </row>
@@ -1033,11 +1033,11 @@
       </c>
       <c r="N5" s="6" t="inlineStr">
         <is>
-          <t>Des 2026</t>
+          <t>Nov 2026</t>
         </is>
       </c>
       <c r="O5" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P5" s="6" t="inlineStr">
         <is>
@@ -1217,11 +1217,11 @@
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>Nov 2026</t>
+          <t>Okt 2026</t>
         </is>
       </c>
       <c r="O7" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
@@ -1308,12 +1308,12 @@
       <c r="L8" s="7" t="inlineStr"/>
       <c r="M8" s="7" t="inlineStr">
         <is>
+          <t>Okt 2026</t>
+        </is>
+      </c>
+      <c r="N8" s="7" t="inlineStr">
+        <is>
           <t>Nov 2026</t>
-        </is>
-      </c>
-      <c r="N8" s="7" t="inlineStr">
-        <is>
-          <t>Des 2026</t>
         </is>
       </c>
       <c r="O8" s="7" t="n">
@@ -1413,11 +1413,11 @@
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>Des 2026</t>
+          <t>Nov 2026</t>
         </is>
       </c>
       <c r="O9" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
@@ -1493,11 +1493,11 @@
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
-          <t>Jan 2027</t>
+          <t>Des 2026</t>
         </is>
       </c>
       <c r="O10" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P10" s="6" t="inlineStr">
         <is>
@@ -1581,11 +1581,11 @@
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>Des 2026</t>
+          <t>Nov 2026</t>
         </is>
       </c>
       <c r="O11" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
@@ -1676,12 +1676,12 @@
       <c r="L12" s="7" t="inlineStr"/>
       <c r="M12" s="7" t="inlineStr">
         <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="N12" s="7" t="inlineStr">
+        <is>
           <t>Des 2026</t>
-        </is>
-      </c>
-      <c r="N12" s="7" t="inlineStr">
-        <is>
-          <t>Jan 2027</t>
         </is>
       </c>
       <c r="O12" s="7" t="n">
@@ -1772,12 +1772,12 @@
       <c r="L13" s="7" t="inlineStr"/>
       <c r="M13" s="7" t="inlineStr">
         <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
           <t>Des 2026</t>
-        </is>
-      </c>
-      <c r="N13" s="7" t="inlineStr">
-        <is>
-          <t>Jan 2027</t>
         </is>
       </c>
       <c r="O13" s="7" t="n">
@@ -1868,12 +1868,12 @@
       <c r="L14" s="7" t="inlineStr"/>
       <c r="M14" s="7" t="inlineStr">
         <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="N14" s="7" t="inlineStr">
+        <is>
           <t>Des 2026</t>
-        </is>
-      </c>
-      <c r="N14" s="7" t="inlineStr">
-        <is>
-          <t>Jan 2027</t>
         </is>
       </c>
       <c r="O14" s="7" t="n">
@@ -1964,12 +1964,12 @@
       <c r="L15" s="7" t="inlineStr"/>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>Jan 2027</t>
+          <t>Des 2026</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>Jan 2027</t>
+          <t>Des 2026</t>
         </is>
       </c>
       <c r="O15" s="7" t="n">
@@ -2044,16 +2044,16 @@
       </c>
       <c r="M16" s="6" t="inlineStr">
         <is>
-          <t>Jan 2027</t>
+          <t>Des 2026</t>
         </is>
       </c>
       <c r="N16" s="6" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>Apr 2027</t>
         </is>
       </c>
       <c r="O16" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="P16" s="6" t="inlineStr">
         <is>
@@ -2132,12 +2132,12 @@
       <c r="L17" s="7" t="inlineStr"/>
       <c r="M17" s="7" t="inlineStr">
         <is>
+          <t>Des 2026</t>
+        </is>
+      </c>
+      <c r="N17" s="7" t="inlineStr">
+        <is>
           <t>Jan 2027</t>
-        </is>
-      </c>
-      <c r="N17" s="7" t="inlineStr">
-        <is>
-          <t>Feb 2027</t>
         </is>
       </c>
       <c r="O17" s="7" t="n">
@@ -2232,16 +2232,16 @@
       <c r="L18" s="7" t="inlineStr"/>
       <c r="M18" s="7" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>Jan 2027</t>
         </is>
       </c>
       <c r="N18" s="7" t="inlineStr">
         <is>
-          <t>Mei 2027</t>
+          <t>Mar 2027</t>
         </is>
       </c>
       <c r="O18" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P18" s="7" t="inlineStr">
         <is>
@@ -2328,16 +2328,16 @@
       <c r="L19" s="7" t="inlineStr"/>
       <c r="M19" s="7" t="inlineStr">
         <is>
+          <t>Jan 2027</t>
+        </is>
+      </c>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
           <t>Feb 2027</t>
         </is>
       </c>
-      <c r="N19" s="7" t="inlineStr">
-        <is>
-          <t>Mei 2027</t>
-        </is>
-      </c>
       <c r="O19" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P19" s="7" t="inlineStr">
         <is>
@@ -2428,16 +2428,16 @@
       <c r="L20" s="7" t="inlineStr"/>
       <c r="M20" s="7" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>Feb 2027</t>
         </is>
       </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>Mei 2027</t>
+          <t>Feb 2027</t>
         </is>
       </c>
       <c r="O20" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P20" s="7" t="inlineStr">
         <is>
@@ -2524,16 +2524,16 @@
       <c r="L21" s="7" t="inlineStr"/>
       <c r="M21" s="7" t="inlineStr">
         <is>
-          <t>Mei 2027</t>
+          <t>Mar 2027</t>
         </is>
       </c>
       <c r="N21" s="7" t="inlineStr">
         <is>
-          <t>Jun 2027</t>
+          <t>Mar 2027</t>
         </is>
       </c>
       <c r="O21" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P21" s="7" t="inlineStr">
         <is>
@@ -2624,12 +2624,12 @@
       <c r="L22" s="7" t="inlineStr"/>
       <c r="M22" s="7" t="inlineStr">
         <is>
-          <t>Jun 2027</t>
+          <t>Mar 2027</t>
         </is>
       </c>
       <c r="N22" s="7" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>Apr 2027</t>
         </is>
       </c>
       <c r="O22" s="7" t="n">
@@ -2720,16 +2720,16 @@
       <c r="L23" s="7" t="inlineStr"/>
       <c r="M23" s="7" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>Jan 2027</t>
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr">
         <is>
-          <t>Jun 2027</t>
+          <t>Mar 2027</t>
         </is>
       </c>
       <c r="O23" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P23" s="7" t="inlineStr">
         <is>
@@ -2796,12 +2796,12 @@
       </c>
       <c r="M24" s="6" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>Jan 2027</t>
         </is>
       </c>
       <c r="N24" s="6" t="inlineStr">
         <is>
-          <t>Sep 2027</t>
+          <t>Jul 2027</t>
         </is>
       </c>
       <c r="O24" s="6" t="n">
@@ -2884,16 +2884,16 @@
       <c r="L25" s="7" t="inlineStr"/>
       <c r="M25" s="7" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>Jan 2027</t>
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>Jun 2027</t>
         </is>
       </c>
       <c r="O25" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P25" s="7" t="inlineStr">
         <is>
@@ -2980,12 +2980,12 @@
       <c r="L26" s="7" t="inlineStr"/>
       <c r="M26" s="7" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>Jan 2027</t>
         </is>
       </c>
       <c r="N26" s="7" t="inlineStr">
         <is>
-          <t>Jun 2027</t>
+          <t>Apr 2027</t>
         </is>
       </c>
       <c r="O26" s="7" t="n">
@@ -3076,12 +3076,12 @@
       <c r="L27" s="7" t="inlineStr"/>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>Feb 2027</t>
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>Mei 2027</t>
         </is>
       </c>
       <c r="O27" s="7" t="n">
@@ -3172,16 +3172,16 @@
       <c r="L28" s="7" t="inlineStr"/>
       <c r="M28" s="7" t="inlineStr">
         <is>
-          <t>Mei 2027</t>
+          <t>Feb 2027</t>
         </is>
       </c>
       <c r="N28" s="7" t="inlineStr">
         <is>
-          <t>Agu 2027</t>
+          <t>Apr 2027</t>
         </is>
       </c>
       <c r="O28" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P28" s="7" t="inlineStr">
         <is>
@@ -3272,16 +3272,16 @@
       <c r="L29" s="7" t="inlineStr"/>
       <c r="M29" s="7" t="inlineStr">
         <is>
+          <t>Apr 2027</t>
+        </is>
+      </c>
+      <c r="N29" s="7" t="inlineStr">
+        <is>
           <t>Jul 2027</t>
         </is>
       </c>
-      <c r="N29" s="7" t="inlineStr">
-        <is>
-          <t>Sep 2027</t>
-        </is>
-      </c>
       <c r="O29" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P29" s="7" t="inlineStr">
         <is>
@@ -3368,12 +3368,12 @@
       <c r="L30" s="7" t="inlineStr"/>
       <c r="M30" s="7" t="inlineStr">
         <is>
-          <t>Mei 2027</t>
+          <t>Mar 2027</t>
         </is>
       </c>
       <c r="N30" s="7" t="inlineStr">
         <is>
-          <t>Sep 2027</t>
+          <t>Jul 2027</t>
         </is>
       </c>
       <c r="O30" s="7" t="n">
@@ -3444,16 +3444,16 @@
       </c>
       <c r="M31" s="6" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>Des 2026</t>
         </is>
       </c>
       <c r="N31" s="6" t="inlineStr">
         <is>
-          <t>Agu 2027</t>
+          <t>Apr 2027</t>
         </is>
       </c>
       <c r="O31" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="P31" s="6" t="inlineStr">
         <is>
@@ -3532,16 +3532,16 @@
       <c r="L32" s="7" t="inlineStr"/>
       <c r="M32" s="7" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>Des 2026</t>
         </is>
       </c>
       <c r="N32" s="7" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>Des 2026</t>
         </is>
       </c>
       <c r="O32" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P32" s="7" t="inlineStr">
         <is>
@@ -3632,16 +3632,16 @@
       <c r="L33" s="7" t="inlineStr"/>
       <c r="M33" s="7" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>Des 2026</t>
         </is>
       </c>
       <c r="N33" s="7" t="inlineStr">
         <is>
-          <t>Mei 2027</t>
+          <t>Jan 2027</t>
         </is>
       </c>
       <c r="O33" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P33" s="7" t="inlineStr">
         <is>
@@ -3732,12 +3732,12 @@
       <c r="L34" s="7" t="inlineStr"/>
       <c r="M34" s="7" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>Jan 2027</t>
         </is>
       </c>
       <c r="N34" s="7" t="inlineStr">
         <is>
-          <t>Mei 2027</t>
+          <t>Feb 2027</t>
         </is>
       </c>
       <c r="O34" s="7" t="n">
@@ -3832,16 +3832,16 @@
       <c r="L35" s="7" t="inlineStr"/>
       <c r="M35" s="7" t="inlineStr">
         <is>
-          <t>Mei 2027</t>
+          <t>Feb 2027</t>
         </is>
       </c>
       <c r="N35" s="7" t="inlineStr">
         <is>
-          <t>Jun 2027</t>
+          <t>Feb 2027</t>
         </is>
       </c>
       <c r="O35" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P35" s="7" t="inlineStr">
         <is>
@@ -3932,12 +3932,12 @@
       <c r="L36" s="7" t="inlineStr"/>
       <c r="M36" s="7" t="inlineStr">
         <is>
-          <t>Jun 2027</t>
+          <t>Feb 2027</t>
         </is>
       </c>
       <c r="N36" s="7" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>Mar 2027</t>
         </is>
       </c>
       <c r="O36" s="7" t="n">
@@ -4032,12 +4032,12 @@
       <c r="L37" s="7" t="inlineStr"/>
       <c r="M37" s="7" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>Mar 2027</t>
         </is>
       </c>
       <c r="N37" s="7" t="inlineStr">
         <is>
-          <t>Agu 2027</t>
+          <t>Apr 2027</t>
         </is>
       </c>
       <c r="O37" s="7" t="n">
@@ -4112,16 +4112,16 @@
       </c>
       <c r="M38" s="6" t="inlineStr">
         <is>
-          <t>Agu 2027</t>
+          <t>Mar 2027</t>
         </is>
       </c>
       <c r="N38" s="6" t="inlineStr">
         <is>
-          <t>Nov 2027</t>
+          <t>Mei 2027</t>
         </is>
       </c>
       <c r="O38" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P38" s="6" t="inlineStr">
         <is>
@@ -4200,12 +4200,12 @@
       <c r="L39" s="7" t="inlineStr"/>
       <c r="M39" s="7" t="inlineStr">
         <is>
-          <t>Agu 2027</t>
+          <t>Mar 2027</t>
         </is>
       </c>
       <c r="N39" s="7" t="inlineStr">
         <is>
-          <t>Agu 2027</t>
+          <t>Mar 2027</t>
         </is>
       </c>
       <c r="O39" s="7" t="n">
@@ -4296,12 +4296,12 @@
       <c r="L40" s="7" t="inlineStr"/>
       <c r="M40" s="7" t="inlineStr">
         <is>
-          <t>Agu 2027</t>
+          <t>Mar 2027</t>
         </is>
       </c>
       <c r="N40" s="7" t="inlineStr">
         <is>
-          <t>Sep 2027</t>
+          <t>Apr 2027</t>
         </is>
       </c>
       <c r="O40" s="7" t="n">
@@ -4396,12 +4396,12 @@
       <c r="L41" s="7" t="inlineStr"/>
       <c r="M41" s="7" t="inlineStr">
         <is>
-          <t>Sep 2027</t>
+          <t>Apr 2027</t>
         </is>
       </c>
       <c r="N41" s="7" t="inlineStr">
         <is>
-          <t>Okt 2027</t>
+          <t>Mei 2027</t>
         </is>
       </c>
       <c r="O41" s="7" t="n">
@@ -4496,16 +4496,16 @@
       <c r="L42" s="7" t="inlineStr"/>
       <c r="M42" s="7" t="inlineStr">
         <is>
-          <t>Jun 2027</t>
+          <t>Jan 2027</t>
         </is>
       </c>
       <c r="N42" s="7" t="inlineStr">
         <is>
-          <t>Sep 2027</t>
+          <t>Mar 2027</t>
         </is>
       </c>
       <c r="O42" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P42" s="7" t="inlineStr">
         <is>
@@ -4592,12 +4592,12 @@
       <c r="L43" s="7" t="inlineStr"/>
       <c r="M43" s="7" t="inlineStr">
         <is>
-          <t>Okt 2027</t>
+          <t>Mei 2027</t>
         </is>
       </c>
       <c r="N43" s="7" t="inlineStr">
         <is>
-          <t>Okt 2027</t>
+          <t>Mei 2027</t>
         </is>
       </c>
       <c r="O43" s="7" t="n">
@@ -4692,12 +4692,12 @@
       <c r="L44" s="7" t="inlineStr"/>
       <c r="M44" s="7" t="inlineStr">
         <is>
-          <t>Nov 2027</t>
+          <t>Mei 2027</t>
         </is>
       </c>
       <c r="N44" s="7" t="inlineStr">
         <is>
-          <t>Nov 2027</t>
+          <t>Mei 2027</t>
         </is>
       </c>
       <c r="O44" s="7" t="n">
@@ -4772,16 +4772,16 @@
       </c>
       <c r="M45" s="6" t="inlineStr">
         <is>
-          <t>Nov 2027</t>
+          <t>Mei 2027</t>
         </is>
       </c>
       <c r="N45" s="6" t="inlineStr">
         <is>
-          <t>Apr 2028</t>
+          <t>Sep 2027</t>
         </is>
       </c>
       <c r="O45" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P45" s="6" t="inlineStr">
         <is>
@@ -4860,16 +4860,16 @@
       <c r="L46" s="7" t="inlineStr"/>
       <c r="M46" s="7" t="inlineStr">
         <is>
-          <t>Nov 2027</t>
+          <t>Mei 2027</t>
         </is>
       </c>
       <c r="N46" s="7" t="inlineStr">
         <is>
-          <t>Jan 2028</t>
+          <t>Jun 2027</t>
         </is>
       </c>
       <c r="O46" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P46" s="7" t="inlineStr">
         <is>
@@ -4960,12 +4960,12 @@
       <c r="L47" s="7" t="inlineStr"/>
       <c r="M47" s="7" t="inlineStr">
         <is>
-          <t>Jan 2028</t>
+          <t>Jun 2027</t>
         </is>
       </c>
       <c r="N47" s="7" t="inlineStr">
         <is>
-          <t>Mar 2028</t>
+          <t>Agu 2027</t>
         </is>
       </c>
       <c r="O47" s="7" t="n">
@@ -5060,12 +5060,12 @@
       <c r="L48" s="7" t="inlineStr"/>
       <c r="M48" s="7" t="inlineStr">
         <is>
-          <t>Jan 2028</t>
+          <t>Jun 2027</t>
         </is>
       </c>
       <c r="N48" s="7" t="inlineStr">
         <is>
-          <t>Mar 2028</t>
+          <t>Agu 2027</t>
         </is>
       </c>
       <c r="O48" s="7" t="n">
@@ -5160,12 +5160,12 @@
       <c r="L49" s="7" t="inlineStr"/>
       <c r="M49" s="7" t="inlineStr">
         <is>
-          <t>Jan 2028</t>
+          <t>Jun 2027</t>
         </is>
       </c>
       <c r="N49" s="7" t="inlineStr">
         <is>
-          <t>Mar 2028</t>
+          <t>Agu 2027</t>
         </is>
       </c>
       <c r="O49" s="7" t="n">
@@ -5256,12 +5256,12 @@
       <c r="L50" s="7" t="inlineStr"/>
       <c r="M50" s="7" t="inlineStr">
         <is>
-          <t>Mar 2028</t>
+          <t>Agu 2027</t>
         </is>
       </c>
       <c r="N50" s="7" t="inlineStr">
         <is>
-          <t>Apr 2028</t>
+          <t>Sep 2027</t>
         </is>
       </c>
       <c r="O50" s="7" t="n">
@@ -5356,12 +5356,12 @@
       <c r="L51" s="7" t="inlineStr"/>
       <c r="M51" s="7" t="inlineStr">
         <is>
-          <t>Apr 2028</t>
+          <t>Sep 2027</t>
         </is>
       </c>
       <c r="N51" s="7" t="inlineStr">
         <is>
-          <t>Apr 2028</t>
+          <t>Sep 2027</t>
         </is>
       </c>
       <c r="O51" s="7" t="n">
@@ -5448,7 +5448,7 @@
       </c>
       <c r="M52" s="8" t="inlineStr">
         <is>
-          <t>2028–2029</t>
+          <t>2027–2029</t>
         </is>
       </c>
       <c r="N52" s="8" t="inlineStr"/>
@@ -5848,7 +5848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V44"/>
+  <dimension ref="A1:R44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5869,10 +5869,6 @@
     <col width="7.5" customWidth="1" min="16" max="16"/>
     <col width="7.5" customWidth="1" min="17" max="17"/>
     <col width="7.5" customWidth="1" min="18" max="18"/>
-    <col width="7.5" customWidth="1" min="19" max="19"/>
-    <col width="7.5" customWidth="1" min="20" max="20"/>
-    <col width="7.5" customWidth="1" min="21" max="21"/>
-    <col width="7.5" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5885,7 +5881,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hijau tua = jalur kritis · hijau muda = ada float · oranye = bergantung review Plan Vivo (indikatif)</t>
+          <t>Hijau tua = jalur kritis · hijau muda = ada float · oranye = bergantung review Plan Vivo · header oranye = setelah TAF berakhir (Sep 2027), buffer review</t>
         </is>
       </c>
     </row>
@@ -5965,12 +5961,12 @@
           <t>Sep 2027</t>
         </is>
       </c>
-      <c r="P4" s="10" t="inlineStr">
+      <c r="P4" s="11" t="inlineStr">
         <is>
           <t>Okt 2027</t>
         </is>
       </c>
-      <c r="Q4" s="10" t="inlineStr">
+      <c r="Q4" s="11" t="inlineStr">
         <is>
           <t>Nov 2027</t>
         </is>
@@ -5978,26 +5974,6 @@
       <c r="R4" s="11" t="inlineStr">
         <is>
           <t>Des 2027</t>
-        </is>
-      </c>
-      <c r="S4" s="11" t="inlineStr">
-        <is>
-          <t>Jan 2028</t>
-        </is>
-      </c>
-      <c r="T4" s="11" t="inlineStr">
-        <is>
-          <t>Feb 2028</t>
-        </is>
-      </c>
-      <c r="U4" s="11" t="inlineStr">
-        <is>
-          <t>Mar 2028</t>
-        </is>
-      </c>
-      <c r="V4" s="11" t="inlineStr">
-        <is>
-          <t>Apr 2028</t>
         </is>
       </c>
     </row>
@@ -6032,10 +6008,6 @@
       <c r="P5" s="14" t="n"/>
       <c r="Q5" s="14" t="n"/>
       <c r="R5" s="14" t="n"/>
-      <c r="S5" s="14" t="n"/>
-      <c r="T5" s="14" t="n"/>
-      <c r="U5" s="14" t="n"/>
-      <c r="V5" s="14" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -6054,7 +6026,7 @@
         </is>
       </c>
       <c r="D6" s="13" t="n"/>
-      <c r="E6" s="13" t="n"/>
+      <c r="E6" s="14" t="n"/>
       <c r="F6" s="14" t="n"/>
       <c r="G6" s="14" t="n"/>
       <c r="H6" s="14" t="n"/>
@@ -6068,10 +6040,6 @@
       <c r="P6" s="14" t="n"/>
       <c r="Q6" s="14" t="n"/>
       <c r="R6" s="14" t="n"/>
-      <c r="S6" s="14" t="n"/>
-      <c r="T6" s="14" t="n"/>
-      <c r="U6" s="14" t="n"/>
-      <c r="V6" s="14" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -6089,9 +6057,9 @@
           <t>PM</t>
         </is>
       </c>
-      <c r="D7" s="14" t="n"/>
+      <c r="D7" s="16" t="n"/>
       <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
+      <c r="F7" s="14" t="n"/>
       <c r="G7" s="14" t="n"/>
       <c r="H7" s="14" t="n"/>
       <c r="I7" s="14" t="n"/>
@@ -6104,10 +6072,6 @@
       <c r="P7" s="14" t="n"/>
       <c r="Q7" s="14" t="n"/>
       <c r="R7" s="14" t="n"/>
-      <c r="S7" s="14" t="n"/>
-      <c r="T7" s="14" t="n"/>
-      <c r="U7" s="14" t="n"/>
-      <c r="V7" s="14" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
@@ -6127,7 +6091,7 @@
       </c>
       <c r="D8" s="16" t="n"/>
       <c r="E8" s="16" t="n"/>
-      <c r="F8" s="16" t="n"/>
+      <c r="F8" s="14" t="n"/>
       <c r="G8" s="14" t="n"/>
       <c r="H8" s="14" t="n"/>
       <c r="I8" s="14" t="n"/>
@@ -6140,10 +6104,6 @@
       <c r="P8" s="14" t="n"/>
       <c r="Q8" s="14" t="n"/>
       <c r="R8" s="14" t="n"/>
-      <c r="S8" s="14" t="n"/>
-      <c r="T8" s="14" t="n"/>
-      <c r="U8" s="14" t="n"/>
-      <c r="V8" s="14" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
@@ -6163,7 +6123,7 @@
       </c>
       <c r="D9" s="14" t="n"/>
       <c r="E9" s="16" t="n"/>
-      <c r="F9" s="16" t="n"/>
+      <c r="F9" s="14" t="n"/>
       <c r="G9" s="14" t="n"/>
       <c r="H9" s="14" t="n"/>
       <c r="I9" s="14" t="n"/>
@@ -6176,10 +6136,6 @@
       <c r="P9" s="14" t="n"/>
       <c r="Q9" s="14" t="n"/>
       <c r="R9" s="14" t="n"/>
-      <c r="S9" s="14" t="n"/>
-      <c r="T9" s="14" t="n"/>
-      <c r="U9" s="14" t="n"/>
-      <c r="V9" s="14" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -6198,9 +6154,9 @@
         </is>
       </c>
       <c r="D10" s="14" t="n"/>
-      <c r="E10" s="14" t="n"/>
+      <c r="E10" s="13" t="n"/>
       <c r="F10" s="13" t="n"/>
-      <c r="G10" s="13" t="n"/>
+      <c r="G10" s="14" t="n"/>
       <c r="H10" s="14" t="n"/>
       <c r="I10" s="14" t="n"/>
       <c r="J10" s="14" t="n"/>
@@ -6212,10 +6168,6 @@
       <c r="P10" s="14" t="n"/>
       <c r="Q10" s="14" t="n"/>
       <c r="R10" s="14" t="n"/>
-      <c r="S10" s="14" t="n"/>
-      <c r="T10" s="14" t="n"/>
-      <c r="U10" s="14" t="n"/>
-      <c r="V10" s="14" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -6234,9 +6186,9 @@
         </is>
       </c>
       <c r="D11" s="14" t="n"/>
-      <c r="E11" s="14" t="n"/>
+      <c r="E11" s="13" t="n"/>
       <c r="F11" s="13" t="n"/>
-      <c r="G11" s="13" t="n"/>
+      <c r="G11" s="14" t="n"/>
       <c r="H11" s="14" t="n"/>
       <c r="I11" s="14" t="n"/>
       <c r="J11" s="14" t="n"/>
@@ -6248,10 +6200,6 @@
       <c r="P11" s="14" t="n"/>
       <c r="Q11" s="14" t="n"/>
       <c r="R11" s="14" t="n"/>
-      <c r="S11" s="14" t="n"/>
-      <c r="T11" s="14" t="n"/>
-      <c r="U11" s="14" t="n"/>
-      <c r="V11" s="14" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -6270,9 +6218,9 @@
         </is>
       </c>
       <c r="D12" s="14" t="n"/>
-      <c r="E12" s="14" t="n"/>
+      <c r="E12" s="13" t="n"/>
       <c r="F12" s="13" t="n"/>
-      <c r="G12" s="13" t="n"/>
+      <c r="G12" s="14" t="n"/>
       <c r="H12" s="14" t="n"/>
       <c r="I12" s="14" t="n"/>
       <c r="J12" s="14" t="n"/>
@@ -6284,10 +6232,6 @@
       <c r="P12" s="14" t="n"/>
       <c r="Q12" s="14" t="n"/>
       <c r="R12" s="14" t="n"/>
-      <c r="S12" s="14" t="n"/>
-      <c r="T12" s="14" t="n"/>
-      <c r="U12" s="14" t="n"/>
-      <c r="V12" s="14" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
@@ -6307,8 +6251,8 @@
       </c>
       <c r="D13" s="14" t="n"/>
       <c r="E13" s="14" t="n"/>
-      <c r="F13" s="14" t="n"/>
-      <c r="G13" s="16" t="n"/>
+      <c r="F13" s="16" t="n"/>
+      <c r="G13" s="14" t="n"/>
       <c r="H13" s="14" t="n"/>
       <c r="I13" s="14" t="n"/>
       <c r="J13" s="14" t="n"/>
@@ -6320,10 +6264,6 @@
       <c r="P13" s="14" t="n"/>
       <c r="Q13" s="14" t="n"/>
       <c r="R13" s="14" t="n"/>
-      <c r="S13" s="14" t="n"/>
-      <c r="T13" s="14" t="n"/>
-      <c r="U13" s="14" t="n"/>
-      <c r="V13" s="14" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
@@ -6343,9 +6283,9 @@
       </c>
       <c r="D14" s="14" t="n"/>
       <c r="E14" s="14" t="n"/>
-      <c r="F14" s="14" t="n"/>
+      <c r="F14" s="16" t="n"/>
       <c r="G14" s="16" t="n"/>
-      <c r="H14" s="16" t="n"/>
+      <c r="H14" s="14" t="n"/>
       <c r="I14" s="14" t="n"/>
       <c r="J14" s="14" t="n"/>
       <c r="K14" s="14" t="n"/>
@@ -6356,10 +6296,6 @@
       <c r="P14" s="14" t="n"/>
       <c r="Q14" s="14" t="n"/>
       <c r="R14" s="14" t="n"/>
-      <c r="S14" s="14" t="n"/>
-      <c r="T14" s="14" t="n"/>
-      <c r="U14" s="14" t="n"/>
-      <c r="V14" s="14" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -6380,11 +6316,11 @@
       <c r="D15" s="14" t="n"/>
       <c r="E15" s="14" t="n"/>
       <c r="F15" s="14" t="n"/>
-      <c r="G15" s="14" t="n"/>
+      <c r="G15" s="13" t="n"/>
       <c r="H15" s="13" t="n"/>
       <c r="I15" s="13" t="n"/>
-      <c r="J15" s="13" t="n"/>
-      <c r="K15" s="13" t="n"/>
+      <c r="J15" s="14" t="n"/>
+      <c r="K15" s="14" t="n"/>
       <c r="L15" s="14" t="n"/>
       <c r="M15" s="14" t="n"/>
       <c r="N15" s="14" t="n"/>
@@ -6392,10 +6328,6 @@
       <c r="P15" s="14" t="n"/>
       <c r="Q15" s="14" t="n"/>
       <c r="R15" s="14" t="n"/>
-      <c r="S15" s="14" t="n"/>
-      <c r="T15" s="14" t="n"/>
-      <c r="U15" s="14" t="n"/>
-      <c r="V15" s="14" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
@@ -6416,11 +6348,11 @@
       <c r="D16" s="14" t="n"/>
       <c r="E16" s="14" t="n"/>
       <c r="F16" s="14" t="n"/>
-      <c r="G16" s="14" t="n"/>
+      <c r="G16" s="16" t="n"/>
       <c r="H16" s="16" t="n"/>
-      <c r="I16" s="16" t="n"/>
-      <c r="J16" s="16" t="n"/>
-      <c r="K16" s="16" t="n"/>
+      <c r="I16" s="14" t="n"/>
+      <c r="J16" s="14" t="n"/>
+      <c r="K16" s="14" t="n"/>
       <c r="L16" s="14" t="n"/>
       <c r="M16" s="14" t="n"/>
       <c r="N16" s="14" t="n"/>
@@ -6428,10 +6360,6 @@
       <c r="P16" s="14" t="n"/>
       <c r="Q16" s="14" t="n"/>
       <c r="R16" s="14" t="n"/>
-      <c r="S16" s="14" t="n"/>
-      <c r="T16" s="14" t="n"/>
-      <c r="U16" s="14" t="n"/>
-      <c r="V16" s="14" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
@@ -6453,10 +6381,10 @@
       <c r="E17" s="14" t="n"/>
       <c r="F17" s="14" t="n"/>
       <c r="G17" s="14" t="n"/>
-      <c r="H17" s="14" t="n"/>
+      <c r="H17" s="13" t="n"/>
       <c r="I17" s="14" t="n"/>
-      <c r="J17" s="13" t="n"/>
-      <c r="K17" s="13" t="n"/>
+      <c r="J17" s="14" t="n"/>
+      <c r="K17" s="14" t="n"/>
       <c r="L17" s="14" t="n"/>
       <c r="M17" s="14" t="n"/>
       <c r="N17" s="14" t="n"/>
@@ -6464,10 +6392,6 @@
       <c r="P17" s="14" t="n"/>
       <c r="Q17" s="14" t="n"/>
       <c r="R17" s="14" t="n"/>
-      <c r="S17" s="14" t="n"/>
-      <c r="T17" s="14" t="n"/>
-      <c r="U17" s="14" t="n"/>
-      <c r="V17" s="14" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
@@ -6490,20 +6414,16 @@
       <c r="F18" s="14" t="n"/>
       <c r="G18" s="14" t="n"/>
       <c r="H18" s="14" t="n"/>
-      <c r="I18" s="14" t="n"/>
+      <c r="I18" s="16" t="n"/>
       <c r="J18" s="14" t="n"/>
-      <c r="K18" s="16" t="n"/>
-      <c r="L18" s="16" t="n"/>
+      <c r="K18" s="14" t="n"/>
+      <c r="L18" s="14" t="n"/>
       <c r="M18" s="14" t="n"/>
       <c r="N18" s="14" t="n"/>
       <c r="O18" s="14" t="n"/>
       <c r="P18" s="14" t="n"/>
       <c r="Q18" s="14" t="n"/>
       <c r="R18" s="14" t="n"/>
-      <c r="S18" s="14" t="n"/>
-      <c r="T18" s="14" t="n"/>
-      <c r="U18" s="14" t="n"/>
-      <c r="V18" s="14" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
@@ -6526,20 +6446,16 @@
       <c r="F19" s="14" t="n"/>
       <c r="G19" s="14" t="n"/>
       <c r="H19" s="14" t="n"/>
-      <c r="I19" s="14" t="n"/>
-      <c r="J19" s="14" t="n"/>
+      <c r="I19" s="13" t="n"/>
+      <c r="J19" s="13" t="n"/>
       <c r="K19" s="14" t="n"/>
-      <c r="L19" s="13" t="n"/>
-      <c r="M19" s="13" t="n"/>
+      <c r="L19" s="14" t="n"/>
+      <c r="M19" s="14" t="n"/>
       <c r="N19" s="14" t="n"/>
       <c r="O19" s="14" t="n"/>
       <c r="P19" s="14" t="n"/>
       <c r="Q19" s="14" t="n"/>
       <c r="R19" s="14" t="n"/>
-      <c r="S19" s="14" t="n"/>
-      <c r="T19" s="14" t="n"/>
-      <c r="U19" s="14" t="n"/>
-      <c r="V19" s="14" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -6560,22 +6476,18 @@
       <c r="D20" s="14" t="n"/>
       <c r="E20" s="14" t="n"/>
       <c r="F20" s="14" t="n"/>
-      <c r="G20" s="14" t="n"/>
+      <c r="G20" s="13" t="n"/>
       <c r="H20" s="13" t="n"/>
       <c r="I20" s="13" t="n"/>
-      <c r="J20" s="13" t="n"/>
-      <c r="K20" s="13" t="n"/>
-      <c r="L20" s="13" t="n"/>
+      <c r="J20" s="14" t="n"/>
+      <c r="K20" s="14" t="n"/>
+      <c r="L20" s="14" t="n"/>
       <c r="M20" s="14" t="n"/>
       <c r="N20" s="14" t="n"/>
       <c r="O20" s="14" t="n"/>
       <c r="P20" s="14" t="n"/>
       <c r="Q20" s="14" t="n"/>
       <c r="R20" s="14" t="n"/>
-      <c r="S20" s="14" t="n"/>
-      <c r="T20" s="14" t="n"/>
-      <c r="U20" s="14" t="n"/>
-      <c r="V20" s="14" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
@@ -6596,22 +6508,18 @@
       <c r="D21" s="14" t="n"/>
       <c r="E21" s="14" t="n"/>
       <c r="F21" s="14" t="n"/>
-      <c r="G21" s="14" t="n"/>
-      <c r="H21" s="14" t="n"/>
+      <c r="G21" s="13" t="n"/>
+      <c r="H21" s="13" t="n"/>
       <c r="I21" s="13" t="n"/>
       <c r="J21" s="13" t="n"/>
       <c r="K21" s="13" t="n"/>
       <c r="L21" s="13" t="n"/>
-      <c r="M21" s="13" t="n"/>
+      <c r="M21" s="14" t="n"/>
       <c r="N21" s="14" t="n"/>
       <c r="O21" s="14" t="n"/>
       <c r="P21" s="14" t="n"/>
       <c r="Q21" s="14" t="n"/>
       <c r="R21" s="14" t="n"/>
-      <c r="S21" s="14" t="n"/>
-      <c r="T21" s="14" t="n"/>
-      <c r="U21" s="14" t="n"/>
-      <c r="V21" s="14" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
@@ -6632,22 +6540,18 @@
       <c r="D22" s="14" t="n"/>
       <c r="E22" s="14" t="n"/>
       <c r="F22" s="14" t="n"/>
-      <c r="G22" s="14" t="n"/>
-      <c r="H22" s="14" t="n"/>
+      <c r="G22" s="13" t="n"/>
+      <c r="H22" s="13" t="n"/>
       <c r="I22" s="13" t="n"/>
       <c r="J22" s="13" t="n"/>
-      <c r="K22" s="13" t="n"/>
-      <c r="L22" s="13" t="n"/>
+      <c r="K22" s="14" t="n"/>
+      <c r="L22" s="14" t="n"/>
       <c r="M22" s="14" t="n"/>
       <c r="N22" s="14" t="n"/>
       <c r="O22" s="14" t="n"/>
       <c r="P22" s="14" t="n"/>
       <c r="Q22" s="14" t="n"/>
       <c r="R22" s="14" t="n"/>
-      <c r="S22" s="14" t="n"/>
-      <c r="T22" s="14" t="n"/>
-      <c r="U22" s="14" t="n"/>
-      <c r="V22" s="14" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
@@ -6669,21 +6573,17 @@
       <c r="E23" s="14" t="n"/>
       <c r="F23" s="14" t="n"/>
       <c r="G23" s="14" t="n"/>
-      <c r="H23" s="14" t="n"/>
-      <c r="I23" s="14" t="n"/>
+      <c r="H23" s="13" t="n"/>
+      <c r="I23" s="13" t="n"/>
       <c r="J23" s="13" t="n"/>
       <c r="K23" s="13" t="n"/>
-      <c r="L23" s="13" t="n"/>
-      <c r="M23" s="13" t="n"/>
+      <c r="L23" s="14" t="n"/>
+      <c r="M23" s="14" t="n"/>
       <c r="N23" s="14" t="n"/>
       <c r="O23" s="14" t="n"/>
       <c r="P23" s="14" t="n"/>
       <c r="Q23" s="14" t="n"/>
       <c r="R23" s="14" t="n"/>
-      <c r="S23" s="14" t="n"/>
-      <c r="T23" s="14" t="n"/>
-      <c r="U23" s="14" t="n"/>
-      <c r="V23" s="14" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
@@ -6705,21 +6605,17 @@
       <c r="E24" s="14" t="n"/>
       <c r="F24" s="14" t="n"/>
       <c r="G24" s="14" t="n"/>
-      <c r="H24" s="14" t="n"/>
-      <c r="I24" s="14" t="n"/>
-      <c r="J24" s="14" t="n"/>
-      <c r="K24" s="16" t="n"/>
-      <c r="L24" s="16" t="n"/>
-      <c r="M24" s="16" t="n"/>
-      <c r="N24" s="16" t="n"/>
+      <c r="H24" s="16" t="n"/>
+      <c r="I24" s="16" t="n"/>
+      <c r="J24" s="16" t="n"/>
+      <c r="K24" s="14" t="n"/>
+      <c r="L24" s="14" t="n"/>
+      <c r="M24" s="14" t="n"/>
+      <c r="N24" s="14" t="n"/>
       <c r="O24" s="14" t="n"/>
       <c r="P24" s="14" t="n"/>
       <c r="Q24" s="14" t="n"/>
       <c r="R24" s="14" t="n"/>
-      <c r="S24" s="14" t="n"/>
-      <c r="T24" s="14" t="n"/>
-      <c r="U24" s="14" t="n"/>
-      <c r="V24" s="14" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
@@ -6743,19 +6639,15 @@
       <c r="G25" s="14" t="n"/>
       <c r="H25" s="14" t="n"/>
       <c r="I25" s="14" t="n"/>
-      <c r="J25" s="14" t="n"/>
-      <c r="K25" s="14" t="n"/>
-      <c r="L25" s="14" t="n"/>
+      <c r="J25" s="13" t="n"/>
+      <c r="K25" s="13" t="n"/>
+      <c r="L25" s="13" t="n"/>
       <c r="M25" s="13" t="n"/>
-      <c r="N25" s="13" t="n"/>
-      <c r="O25" s="13" t="n"/>
+      <c r="N25" s="14" t="n"/>
+      <c r="O25" s="14" t="n"/>
       <c r="P25" s="14" t="n"/>
       <c r="Q25" s="14" t="n"/>
       <c r="R25" s="14" t="n"/>
-      <c r="S25" s="14" t="n"/>
-      <c r="T25" s="14" t="n"/>
-      <c r="U25" s="14" t="n"/>
-      <c r="V25" s="14" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
@@ -6778,20 +6670,16 @@
       <c r="F26" s="14" t="n"/>
       <c r="G26" s="14" t="n"/>
       <c r="H26" s="14" t="n"/>
-      <c r="I26" s="14" t="n"/>
-      <c r="J26" s="14" t="n"/>
+      <c r="I26" s="13" t="n"/>
+      <c r="J26" s="13" t="n"/>
       <c r="K26" s="13" t="n"/>
       <c r="L26" s="13" t="n"/>
       <c r="M26" s="13" t="n"/>
-      <c r="N26" s="13" t="n"/>
-      <c r="O26" s="13" t="n"/>
+      <c r="N26" s="14" t="n"/>
+      <c r="O26" s="14" t="n"/>
       <c r="P26" s="14" t="n"/>
       <c r="Q26" s="14" t="n"/>
       <c r="R26" s="14" t="n"/>
-      <c r="S26" s="14" t="n"/>
-      <c r="T26" s="14" t="n"/>
-      <c r="U26" s="14" t="n"/>
-      <c r="V26" s="14" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
@@ -6811,10 +6699,10 @@
       </c>
       <c r="D27" s="14" t="n"/>
       <c r="E27" s="14" t="n"/>
-      <c r="F27" s="14" t="n"/>
+      <c r="F27" s="16" t="n"/>
       <c r="G27" s="14" t="n"/>
-      <c r="H27" s="16" t="n"/>
-      <c r="I27" s="16" t="n"/>
+      <c r="H27" s="14" t="n"/>
+      <c r="I27" s="14" t="n"/>
       <c r="J27" s="14" t="n"/>
       <c r="K27" s="14" t="n"/>
       <c r="L27" s="14" t="n"/>
@@ -6824,10 +6712,6 @@
       <c r="P27" s="14" t="n"/>
       <c r="Q27" s="14" t="n"/>
       <c r="R27" s="14" t="n"/>
-      <c r="S27" s="14" t="n"/>
-      <c r="T27" s="14" t="n"/>
-      <c r="U27" s="14" t="n"/>
-      <c r="V27" s="14" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
@@ -6847,12 +6731,12 @@
       </c>
       <c r="D28" s="14" t="n"/>
       <c r="E28" s="14" t="n"/>
-      <c r="F28" s="14" t="n"/>
-      <c r="G28" s="14" t="n"/>
+      <c r="F28" s="16" t="n"/>
+      <c r="G28" s="16" t="n"/>
       <c r="H28" s="14" t="n"/>
-      <c r="I28" s="16" t="n"/>
-      <c r="J28" s="16" t="n"/>
-      <c r="K28" s="16" t="n"/>
+      <c r="I28" s="14" t="n"/>
+      <c r="J28" s="14" t="n"/>
+      <c r="K28" s="14" t="n"/>
       <c r="L28" s="14" t="n"/>
       <c r="M28" s="14" t="n"/>
       <c r="N28" s="14" t="n"/>
@@ -6860,10 +6744,6 @@
       <c r="P28" s="14" t="n"/>
       <c r="Q28" s="14" t="n"/>
       <c r="R28" s="14" t="n"/>
-      <c r="S28" s="14" t="n"/>
-      <c r="T28" s="14" t="n"/>
-      <c r="U28" s="14" t="n"/>
-      <c r="V28" s="14" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
@@ -6884,11 +6764,11 @@
       <c r="D29" s="14" t="n"/>
       <c r="E29" s="14" t="n"/>
       <c r="F29" s="14" t="n"/>
-      <c r="G29" s="14" t="n"/>
-      <c r="H29" s="14" t="n"/>
+      <c r="G29" s="16" t="n"/>
+      <c r="H29" s="16" t="n"/>
       <c r="I29" s="14" t="n"/>
-      <c r="J29" s="16" t="n"/>
-      <c r="K29" s="16" t="n"/>
+      <c r="J29" s="14" t="n"/>
+      <c r="K29" s="14" t="n"/>
       <c r="L29" s="14" t="n"/>
       <c r="M29" s="14" t="n"/>
       <c r="N29" s="14" t="n"/>
@@ -6896,10 +6776,6 @@
       <c r="P29" s="14" t="n"/>
       <c r="Q29" s="14" t="n"/>
       <c r="R29" s="14" t="n"/>
-      <c r="S29" s="14" t="n"/>
-      <c r="T29" s="14" t="n"/>
-      <c r="U29" s="14" t="n"/>
-      <c r="V29" s="14" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="15" t="inlineStr">
@@ -6921,21 +6797,17 @@
       <c r="E30" s="14" t="n"/>
       <c r="F30" s="14" t="n"/>
       <c r="G30" s="14" t="n"/>
-      <c r="H30" s="14" t="n"/>
+      <c r="H30" s="16" t="n"/>
       <c r="I30" s="14" t="n"/>
       <c r="J30" s="14" t="n"/>
-      <c r="K30" s="16" t="n"/>
-      <c r="L30" s="16" t="n"/>
+      <c r="K30" s="14" t="n"/>
+      <c r="L30" s="14" t="n"/>
       <c r="M30" s="14" t="n"/>
       <c r="N30" s="14" t="n"/>
       <c r="O30" s="14" t="n"/>
       <c r="P30" s="14" t="n"/>
       <c r="Q30" s="14" t="n"/>
       <c r="R30" s="14" t="n"/>
-      <c r="S30" s="14" t="n"/>
-      <c r="T30" s="14" t="n"/>
-      <c r="U30" s="14" t="n"/>
-      <c r="V30" s="14" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="15" t="inlineStr">
@@ -6957,21 +6829,17 @@
       <c r="E31" s="14" t="n"/>
       <c r="F31" s="14" t="n"/>
       <c r="G31" s="14" t="n"/>
-      <c r="H31" s="14" t="n"/>
-      <c r="I31" s="14" t="n"/>
+      <c r="H31" s="16" t="n"/>
+      <c r="I31" s="16" t="n"/>
       <c r="J31" s="14" t="n"/>
       <c r="K31" s="14" t="n"/>
-      <c r="L31" s="16" t="n"/>
-      <c r="M31" s="16" t="n"/>
+      <c r="L31" s="14" t="n"/>
+      <c r="M31" s="14" t="n"/>
       <c r="N31" s="14" t="n"/>
       <c r="O31" s="14" t="n"/>
       <c r="P31" s="14" t="n"/>
       <c r="Q31" s="14" t="n"/>
       <c r="R31" s="14" t="n"/>
-      <c r="S31" s="14" t="n"/>
-      <c r="T31" s="14" t="n"/>
-      <c r="U31" s="14" t="n"/>
-      <c r="V31" s="14" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="15" t="inlineStr">
@@ -6994,20 +6862,16 @@
       <c r="F32" s="14" t="n"/>
       <c r="G32" s="14" t="n"/>
       <c r="H32" s="14" t="n"/>
-      <c r="I32" s="14" t="n"/>
-      <c r="J32" s="14" t="n"/>
+      <c r="I32" s="16" t="n"/>
+      <c r="J32" s="16" t="n"/>
       <c r="K32" s="14" t="n"/>
       <c r="L32" s="14" t="n"/>
-      <c r="M32" s="16" t="n"/>
-      <c r="N32" s="16" t="n"/>
+      <c r="M32" s="14" t="n"/>
+      <c r="N32" s="14" t="n"/>
       <c r="O32" s="14" t="n"/>
       <c r="P32" s="14" t="n"/>
       <c r="Q32" s="14" t="n"/>
       <c r="R32" s="14" t="n"/>
-      <c r="S32" s="14" t="n"/>
-      <c r="T32" s="14" t="n"/>
-      <c r="U32" s="14" t="n"/>
-      <c r="V32" s="14" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
@@ -7030,20 +6894,16 @@
       <c r="F33" s="14" t="n"/>
       <c r="G33" s="14" t="n"/>
       <c r="H33" s="14" t="n"/>
-      <c r="I33" s="14" t="n"/>
+      <c r="I33" s="13" t="n"/>
       <c r="J33" s="14" t="n"/>
       <c r="K33" s="14" t="n"/>
       <c r="L33" s="14" t="n"/>
       <c r="M33" s="14" t="n"/>
-      <c r="N33" s="13" t="n"/>
+      <c r="N33" s="14" t="n"/>
       <c r="O33" s="14" t="n"/>
       <c r="P33" s="14" t="n"/>
       <c r="Q33" s="14" t="n"/>
       <c r="R33" s="14" t="n"/>
-      <c r="S33" s="14" t="n"/>
-      <c r="T33" s="14" t="n"/>
-      <c r="U33" s="14" t="n"/>
-      <c r="V33" s="14" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
@@ -7066,20 +6926,16 @@
       <c r="F34" s="14" t="n"/>
       <c r="G34" s="14" t="n"/>
       <c r="H34" s="14" t="n"/>
-      <c r="I34" s="14" t="n"/>
-      <c r="J34" s="14" t="n"/>
+      <c r="I34" s="16" t="n"/>
+      <c r="J34" s="16" t="n"/>
       <c r="K34" s="14" t="n"/>
       <c r="L34" s="14" t="n"/>
       <c r="M34" s="14" t="n"/>
-      <c r="N34" s="16" t="n"/>
-      <c r="O34" s="16" t="n"/>
+      <c r="N34" s="14" t="n"/>
+      <c r="O34" s="14" t="n"/>
       <c r="P34" s="14" t="n"/>
       <c r="Q34" s="14" t="n"/>
       <c r="R34" s="14" t="n"/>
-      <c r="S34" s="14" t="n"/>
-      <c r="T34" s="14" t="n"/>
-      <c r="U34" s="14" t="n"/>
-      <c r="V34" s="14" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="15" t="inlineStr">
@@ -7103,19 +6959,15 @@
       <c r="G35" s="14" t="n"/>
       <c r="H35" s="14" t="n"/>
       <c r="I35" s="14" t="n"/>
-      <c r="J35" s="14" t="n"/>
-      <c r="K35" s="14" t="n"/>
+      <c r="J35" s="16" t="n"/>
+      <c r="K35" s="16" t="n"/>
       <c r="L35" s="14" t="n"/>
       <c r="M35" s="14" t="n"/>
       <c r="N35" s="14" t="n"/>
-      <c r="O35" s="16" t="n"/>
-      <c r="P35" s="16" t="n"/>
+      <c r="O35" s="14" t="n"/>
+      <c r="P35" s="14" t="n"/>
       <c r="Q35" s="14" t="n"/>
       <c r="R35" s="14" t="n"/>
-      <c r="S35" s="14" t="n"/>
-      <c r="T35" s="14" t="n"/>
-      <c r="U35" s="14" t="n"/>
-      <c r="V35" s="14" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
@@ -7136,22 +6988,18 @@
       <c r="D36" s="14" t="n"/>
       <c r="E36" s="14" t="n"/>
       <c r="F36" s="14" t="n"/>
-      <c r="G36" s="14" t="n"/>
-      <c r="H36" s="14" t="n"/>
-      <c r="I36" s="14" t="n"/>
+      <c r="G36" s="13" t="n"/>
+      <c r="H36" s="13" t="n"/>
+      <c r="I36" s="13" t="n"/>
       <c r="J36" s="14" t="n"/>
       <c r="K36" s="14" t="n"/>
-      <c r="L36" s="13" t="n"/>
-      <c r="M36" s="13" t="n"/>
-      <c r="N36" s="13" t="n"/>
-      <c r="O36" s="13" t="n"/>
+      <c r="L36" s="14" t="n"/>
+      <c r="M36" s="14" t="n"/>
+      <c r="N36" s="14" t="n"/>
+      <c r="O36" s="14" t="n"/>
       <c r="P36" s="14" t="n"/>
       <c r="Q36" s="14" t="n"/>
       <c r="R36" s="14" t="n"/>
-      <c r="S36" s="14" t="n"/>
-      <c r="T36" s="14" t="n"/>
-      <c r="U36" s="14" t="n"/>
-      <c r="V36" s="14" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="15" t="inlineStr">
@@ -7176,18 +7024,14 @@
       <c r="H37" s="14" t="n"/>
       <c r="I37" s="14" t="n"/>
       <c r="J37" s="14" t="n"/>
-      <c r="K37" s="14" t="n"/>
+      <c r="K37" s="16" t="n"/>
       <c r="L37" s="14" t="n"/>
       <c r="M37" s="14" t="n"/>
       <c r="N37" s="14" t="n"/>
       <c r="O37" s="14" t="n"/>
-      <c r="P37" s="16" t="n"/>
+      <c r="P37" s="14" t="n"/>
       <c r="Q37" s="14" t="n"/>
       <c r="R37" s="14" t="n"/>
-      <c r="S37" s="14" t="n"/>
-      <c r="T37" s="14" t="n"/>
-      <c r="U37" s="14" t="n"/>
-      <c r="V37" s="14" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="15" t="inlineStr">
@@ -7212,18 +7056,14 @@
       <c r="H38" s="14" t="n"/>
       <c r="I38" s="14" t="n"/>
       <c r="J38" s="14" t="n"/>
-      <c r="K38" s="14" t="n"/>
+      <c r="K38" s="16" t="n"/>
       <c r="L38" s="14" t="n"/>
       <c r="M38" s="14" t="n"/>
       <c r="N38" s="14" t="n"/>
       <c r="O38" s="14" t="n"/>
       <c r="P38" s="14" t="n"/>
-      <c r="Q38" s="16" t="n"/>
+      <c r="Q38" s="14" t="n"/>
       <c r="R38" s="14" t="n"/>
-      <c r="S38" s="14" t="n"/>
-      <c r="T38" s="14" t="n"/>
-      <c r="U38" s="14" t="n"/>
-      <c r="V38" s="14" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="15" t="inlineStr">
@@ -7248,18 +7088,14 @@
       <c r="H39" s="14" t="n"/>
       <c r="I39" s="14" t="n"/>
       <c r="J39" s="14" t="n"/>
-      <c r="K39" s="14" t="n"/>
-      <c r="L39" s="14" t="n"/>
+      <c r="K39" s="17" t="n"/>
+      <c r="L39" s="17" t="n"/>
       <c r="M39" s="14" t="n"/>
       <c r="N39" s="14" t="n"/>
       <c r="O39" s="14" t="n"/>
       <c r="P39" s="14" t="n"/>
-      <c r="Q39" s="17" t="n"/>
-      <c r="R39" s="17" t="n"/>
-      <c r="S39" s="17" t="n"/>
-      <c r="T39" s="14" t="n"/>
-      <c r="U39" s="14" t="n"/>
-      <c r="V39" s="14" t="n"/>
+      <c r="Q39" s="14" t="n"/>
+      <c r="R39" s="14" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="15" t="inlineStr">
@@ -7285,17 +7121,13 @@
       <c r="I40" s="14" t="n"/>
       <c r="J40" s="14" t="n"/>
       <c r="K40" s="14" t="n"/>
-      <c r="L40" s="14" t="n"/>
-      <c r="M40" s="14" t="n"/>
-      <c r="N40" s="14" t="n"/>
+      <c r="L40" s="17" t="n"/>
+      <c r="M40" s="17" t="n"/>
+      <c r="N40" s="17" t="n"/>
       <c r="O40" s="14" t="n"/>
       <c r="P40" s="14" t="n"/>
       <c r="Q40" s="14" t="n"/>
       <c r="R40" s="14" t="n"/>
-      <c r="S40" s="17" t="n"/>
-      <c r="T40" s="17" t="n"/>
-      <c r="U40" s="17" t="n"/>
-      <c r="V40" s="14" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="15" t="inlineStr">
@@ -7321,17 +7153,13 @@
       <c r="I41" s="14" t="n"/>
       <c r="J41" s="14" t="n"/>
       <c r="K41" s="14" t="n"/>
-      <c r="L41" s="14" t="n"/>
-      <c r="M41" s="14" t="n"/>
-      <c r="N41" s="14" t="n"/>
+      <c r="L41" s="17" t="n"/>
+      <c r="M41" s="17" t="n"/>
+      <c r="N41" s="17" t="n"/>
       <c r="O41" s="14" t="n"/>
       <c r="P41" s="14" t="n"/>
       <c r="Q41" s="14" t="n"/>
       <c r="R41" s="14" t="n"/>
-      <c r="S41" s="17" t="n"/>
-      <c r="T41" s="17" t="n"/>
-      <c r="U41" s="17" t="n"/>
-      <c r="V41" s="14" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="12" t="inlineStr">
@@ -7357,17 +7185,13 @@
       <c r="I42" s="14" t="n"/>
       <c r="J42" s="14" t="n"/>
       <c r="K42" s="14" t="n"/>
-      <c r="L42" s="14" t="n"/>
-      <c r="M42" s="14" t="n"/>
-      <c r="N42" s="14" t="n"/>
+      <c r="L42" s="17" t="n"/>
+      <c r="M42" s="17" t="n"/>
+      <c r="N42" s="17" t="n"/>
       <c r="O42" s="14" t="n"/>
       <c r="P42" s="14" t="n"/>
       <c r="Q42" s="14" t="n"/>
       <c r="R42" s="14" t="n"/>
-      <c r="S42" s="17" t="n"/>
-      <c r="T42" s="17" t="n"/>
-      <c r="U42" s="17" t="n"/>
-      <c r="V42" s="14" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="15" t="inlineStr">
@@ -7395,15 +7219,11 @@
       <c r="K43" s="14" t="n"/>
       <c r="L43" s="14" t="n"/>
       <c r="M43" s="14" t="n"/>
-      <c r="N43" s="14" t="n"/>
-      <c r="O43" s="14" t="n"/>
+      <c r="N43" s="17" t="n"/>
+      <c r="O43" s="17" t="n"/>
       <c r="P43" s="14" t="n"/>
       <c r="Q43" s="14" t="n"/>
       <c r="R43" s="14" t="n"/>
-      <c r="S43" s="14" t="n"/>
-      <c r="T43" s="14" t="n"/>
-      <c r="U43" s="17" t="n"/>
-      <c r="V43" s="17" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="12" t="inlineStr">
@@ -7432,14 +7252,10 @@
       <c r="L44" s="14" t="n"/>
       <c r="M44" s="14" t="n"/>
       <c r="N44" s="14" t="n"/>
-      <c r="O44" s="14" t="n"/>
+      <c r="O44" s="17" t="n"/>
       <c r="P44" s="14" t="n"/>
       <c r="Q44" s="14" t="n"/>
       <c r="R44" s="14" t="n"/>
-      <c r="S44" s="14" t="n"/>
-      <c r="T44" s="14" t="n"/>
-      <c r="U44" s="14" t="n"/>
-      <c r="V44" s="17" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8896,7 +8712,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Sedang</t>
+          <t>Tinggi</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -8906,7 +8722,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Mulai pra-FPIC di bulan 4; buffer 1–2 bulan; PIN dapat disusun paralel tapi tidak dikirim sebelum BA FPIC i–ii</t>
+          <t>Mulai pra-FPIC di bulan 3; jadwal FPIC 4 bulan sangat ketat — jangan dipaksa; PIN disusun paralel tapi tidak dikirim sebelum BA FPIC i–ii</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -9116,7 +8932,7 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Kontrak tenaga ahli sejak bulan 5; transfer pengetahuan ke tim SAMPAN</t>
+          <t>Kontrak tenaga ahli sejak bulan 2; transfer pengetahuan ke tim SAMPAN</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -9138,7 +8954,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Program SETAPAK 4 berakhir sebelum Plan Vivo memberi keputusan</t>
+          <t>TAF berakhir Sep 2027 sebelum Plan Vivo memberi keputusan PIN</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -9148,17 +8964,17 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Sedang</t>
+          <t>Tinggi</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Sedang</t>
+          <t>Tinggi</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Kirim PIN ≤bulan 14; anggarkan tindak lanjut review; handover ke pendanaan lanjutan</t>
+          <t>Kirim PIN ≤Mei 2027 (bulan 8); tanggapi CAR/NIR ≤2 minggu; sepakati dengan TAF indikator 'PIN submitted' + acceptance sebagai target; siapkan anggaran/no-cost extension untuk tindak lanjut review Okt–Des 2027</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Move SETAPAK 4 gate after stage 3: pipeline entry is the programme's main output
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tt9bQwcKRKX4vaP5NybJqL
</commit_message>
<xml_diff>
--- a/hutan-desa-pasir/Milestone_Matrix_HD_Pasir_PVClimate.xlsx
+++ b/hutan-desa-pasir/Milestone_Matrix_HD_Pasir_PVClimate.xlsx
@@ -6042,7 +6042,7 @@
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>Tahap 3 — Masuk Pipeline PV &amp; Mobilisasi Investasi</t>
+          <t>Tahap 3 — Masuk Pipeline PV (Output Utama SETAPAK 4)</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
@@ -8105,7 +8105,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tahap 1–2 = SETAPAK 4 · Tahap 3 = gerbang pipeline &amp; investasi · Tahap 4–8 = pengembangan lanjutan</t>
+          <t>Tahap 1–3 = SETAPAK 4 (Tahap 3 = output utama: masuk Pipeline PV) · Tahap 4–8 = pengembangan lanjutan</t>
         </is>
       </c>
     </row>
@@ -8207,27 +8207,27 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Masuk Pipeline PV &amp; Mobilisasi Investasi</t>
+          <t>Masuk Pipeline PV (Output Utama SETAPAK 4)</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>M7.5 · M8</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Sep 2027 – 2028</t>
+          <t>Sep 2027</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Transisi</t>
+          <t>SETAPAK 4</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>PIN dipublikasikan di pipeline Plan Vivo; Investor/offtaker: pre-financing &amp; kontrak offtake berjangka (presale); Pendamping teregistrasi &amp; pencatatan DPP (Permenhut 6/2026)</t>
+          <t>Output utama SETAPAK 4: PIN disetujui, proyek tercantum &amp; dipublikasikan di pipeline Plan Vivo; Profil proyek &amp; penjajakan investor/offtaker dimulai; pre-financing/presale berjangka berlanjut di STEP 2; Status pendamping teregistrasi &amp; rencana pencatatan DPP (Permenhut 6/2026)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Switch slides to Open Sauce Sans and bundle the font (OFL)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tt9bQwcKRKX4vaP5NybJqL
</commit_message>
<xml_diff>
--- a/hutan-desa-pasir/Milestone_Matrix_HD_Pasir_PVClimate.xlsx
+++ b/hutan-desa-pasir/Milestone_Matrix_HD_Pasir_PVClimate.xlsx
@@ -6089,7 +6089,7 @@
       </c>
       <c r="N54" s="8" t="inlineStr">
         <is>
-          <t>Sep 2027 – 2028</t>
+          <t>2027–2028</t>
         </is>
       </c>
       <c r="O54" s="8" t="inlineStr"/>
@@ -6116,7 +6116,7 @@
       </c>
       <c r="W54" s="8" t="inlineStr">
         <is>
-          <t>Presale: Permenhut 6/2026 Ps. 10(1) mensyaratkan kepemilikan Unit Karbon untuk perdagangan → kontrak berjangka, bukan penjualan unit; konfirmasi hukum</t>
+          <t>Presale = kontrak berjangka (Permenhut 6/2026 Ps. 10(1): dagang butuh Unit Karbon); konfirmasi hukum</t>
         </is>
       </c>
     </row>
@@ -10318,7 +10318,7 @@
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>Presale: Permenhut 6/2026 Ps. 10(1) mensyaratkan kepemilikan Unit Karbon untuk perdagangan → kontrak berjangka, bukan penjualan unit; konfirmasi hukum</t>
+          <t>Presale = kontrak berjangka (Permenhut 6/2026 Ps. 10(1): dagang butuh Unit Karbon); konfirmasi hukum</t>
         </is>
       </c>
     </row>

</xml_diff>